<commit_message>
Se configura kit mantención yamalube semim 10w40 con filtro hibari
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="OMITIDOS" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="196">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -607,6 +607,15 @@
   </si>
   <si>
     <t>MLC4229052730</t>
+  </si>
+  <si>
+    <t>MLC4460683786</t>
+  </si>
+  <si>
+    <t>MLC4414859068</t>
+  </si>
+  <si>
+    <t>MLC4410899690</t>
   </si>
 </sst>
 </file>
@@ -1193,7 +1202,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
@@ -1588,6 +1597,22 @@
       </c>
       <c r="B48" t="s">
         <v>189</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>193</v>
+      </c>
+      <c r="B49" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>193</v>
+      </c>
+      <c r="B50" t="s">
+        <v>195</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se configura kit yamalube semi + filtro hibari
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="197">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -616,6 +616,9 @@
   </si>
   <si>
     <t>MLC4410899690</t>
+  </si>
+  <si>
+    <t>MLC4480631960</t>
   </si>
 </sst>
 </file>
@@ -1202,7 +1205,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:C50"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
@@ -1612,6 +1615,22 @@
         <v>193</v>
       </c>
       <c r="B50" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>196</v>
+      </c>
+      <c r="B51" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>196</v>
+      </c>
+      <c r="B52" t="s">
         <v>195</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Se configura kit yamalube full + filtro fz15
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="199">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -619,6 +619,12 @@
   </si>
   <si>
     <t>MLC4480631960</t>
+  </si>
+  <si>
+    <t>MLC4460707724</t>
+  </si>
+  <si>
+    <t>MLC1658552283</t>
   </si>
 </sst>
 </file>
@@ -1205,7 +1211,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:C52"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
@@ -1632,6 +1638,22 @@
       </c>
       <c r="B52" t="s">
         <v>195</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>197</v>
+      </c>
+      <c r="B53" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>197</v>
+      </c>
+      <c r="B54" t="s">
+        <v>198</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se configura par bujías cr8eix
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="OMITIDOS" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="200">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -625,6 +625,9 @@
   </si>
   <si>
     <t>MLC1658552283</t>
+  </si>
+  <si>
+    <t>MLC2228230541</t>
   </si>
 </sst>
 </file>
@@ -1674,7 +1677,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
@@ -2108,6 +2111,17 @@
       </c>
       <c r="C48">
         <v>6</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>199</v>
+      </c>
+      <c r="B49">
+        <v>4</v>
+      </c>
+      <c r="C49">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se configura mínimo Castrol Power 1 10w50
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="201">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -628,6 +628,9 @@
   </si>
   <si>
     <t>MLC2228230541</t>
+  </si>
+  <si>
+    <t>MLC3968099764</t>
   </si>
 </sst>
 </file>
@@ -1677,7 +1680,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
@@ -2122,6 +2125,14 @@
       </c>
       <c r="C49">
         <v>2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>200</v>
+      </c>
+      <c r="B50">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se omiten publicaciones de catálogo
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648"/>
   </bookViews>
   <sheets>
     <sheet name="OMITIDOS" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="204">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -631,6 +631,15 @@
   </si>
   <si>
     <t>MLC3968099764</t>
+  </si>
+  <si>
+    <t>MLC4417751620</t>
+  </si>
+  <si>
+    <t>MLC3942015756</t>
+  </si>
+  <si>
+    <t>MLC3965088378</t>
   </si>
 </sst>
 </file>
@@ -956,7 +965,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A49"/>
+  <dimension ref="A1:A52"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" style="1" bestFit="1" customWidth="1"/>
@@ -1205,6 +1214,21 @@
     <row r="49" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
         <v>168</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A50" s="1" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A51" s="1" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A52" s="1" t="s">
+        <v>203</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se configuran publicaciones de catalógo
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="OMITIDOS" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">OMITIDOS!$A$1:$A$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Pack!$A$1:$B$42</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stock ML'!$A$1:$B$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stock ML'!$A$1:$B$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'VARIANTES VALIDAR'!$A$1:$A$54</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="205">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -640,6 +640,9 @@
   </si>
   <si>
     <t>MLC3965088378</t>
+  </si>
+  <si>
+    <t>MLC4006471046</t>
   </si>
 </sst>
 </file>
@@ -965,7 +968,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A52"/>
+  <dimension ref="A1:A54"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" style="1" bestFit="1" customWidth="1"/>
@@ -1229,6 +1232,16 @@
     <row r="52" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
         <v>203</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A53" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A54" s="1" t="s">
+        <v>204</v>
       </c>
     </row>
   </sheetData>
@@ -1704,7 +1717,8 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C50"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
@@ -1722,7 +1736,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -1730,7 +1744,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -1738,7 +1752,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -1746,7 +1760,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1754,52 +1768,52 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B6">
-        <v>9</v>
-      </c>
-      <c r="C6">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10">
+        <v>6</v>
+      </c>
+      <c r="C10">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B11">
         <v>6</v>
@@ -1808,9 +1822,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B12">
         <v>6</v>
@@ -1821,346 +1835,341 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B13">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C13">
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B14">
         <v>6</v>
       </c>
-      <c r="C14">
+    </row>
+    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>34</v>
+      </c>
+      <c r="B20">
+        <v>6</v>
+      </c>
+      <c r="C20">
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>27</v>
-      </c>
-      <c r="B15">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>28</v>
-      </c>
-      <c r="B16">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
-        <v>29</v>
-      </c>
-      <c r="B17">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>30</v>
-      </c>
-      <c r="B18">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>31</v>
-      </c>
-      <c r="B19">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>32</v>
-      </c>
-      <c r="B20">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B21">
         <v>6</v>
       </c>
-      <c r="C21">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    </row>
+    <row r="22" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B22">
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B23">
         <v>6</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B24">
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B25">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B26">
         <v>4</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="C26">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B27">
         <v>4</v>
       </c>
-      <c r="C27">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    </row>
+    <row r="28" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B28">
         <v>4</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B29">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30">
+        <v>6</v>
+      </c>
+      <c r="C30">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>155</v>
+      </c>
+      <c r="B31">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>159</v>
+      </c>
+      <c r="B32">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>160</v>
+      </c>
+      <c r="B33">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>162</v>
+      </c>
+      <c r="B34">
+        <v>6</v>
+      </c>
+      <c r="C34">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>170</v>
+      </c>
+      <c r="B35">
+        <v>6</v>
+      </c>
+      <c r="C35">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>171</v>
+      </c>
+      <c r="B36">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>172</v>
+      </c>
+      <c r="B37">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>173</v>
+      </c>
+      <c r="B38">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>174</v>
+      </c>
+      <c r="B39">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>175</v>
+      </c>
+      <c r="B40">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>176</v>
+      </c>
+      <c r="B41">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>177</v>
+      </c>
+      <c r="B42">
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>43</v>
-      </c>
-      <c r="B30">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>32</v>
-      </c>
-      <c r="B31">
-        <v>6</v>
-      </c>
-      <c r="C31">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>155</v>
-      </c>
-      <c r="B32">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>159</v>
-      </c>
-      <c r="B33">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>160</v>
-      </c>
-      <c r="B34">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>162</v>
-      </c>
-      <c r="B35">
-        <v>6</v>
-      </c>
-      <c r="C35">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
-        <v>170</v>
-      </c>
-      <c r="B36">
-        <v>6</v>
-      </c>
-      <c r="C36">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
-        <v>171</v>
-      </c>
-      <c r="B37">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
-        <v>172</v>
-      </c>
-      <c r="B38">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
-        <v>173</v>
-      </c>
-      <c r="B39">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
-        <v>174</v>
-      </c>
-      <c r="B40">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
-        <v>175</v>
-      </c>
-      <c r="B41">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A42" t="s">
-        <v>176</v>
-      </c>
-      <c r="B42">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>177</v>
+        <v>15</v>
       </c>
       <c r="B43">
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>15</v>
+        <v>178</v>
       </c>
       <c r="B44">
+        <v>14</v>
+      </c>
+      <c r="C44">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>179</v>
+      </c>
+      <c r="B45">
+        <v>12</v>
+      </c>
+      <c r="C45">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>181</v>
+      </c>
+      <c r="B46">
+        <v>8</v>
+      </c>
+      <c r="C46">
         <v>4</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A45" t="s">
-        <v>178</v>
-      </c>
-      <c r="B45">
-        <v>14</v>
-      </c>
-      <c r="C45">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A46" t="s">
-        <v>179</v>
-      </c>
-      <c r="B46">
+    <row r="47" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>192</v>
+      </c>
+      <c r="B47">
         <v>12</v>
       </c>
-      <c r="C46">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A47" t="s">
-        <v>181</v>
-      </c>
-      <c r="B47">
-        <v>8</v>
-      </c>
       <c r="C47">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>199</v>
+      </c>
+      <c r="B48">
         <v>4</v>
       </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A48" t="s">
-        <v>192</v>
-      </c>
-      <c r="B48">
-        <v>12</v>
-      </c>
       <c r="C48">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B49">
         <v>4</v>
       </c>
-      <c r="C49">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A50" t="s">
-        <v>200</v>
-      </c>
-      <c r="B50">
-        <v>4</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B47"/>
+  <autoFilter ref="A1:B49">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="MLC3394755938"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="260" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Se configuran publicaciones de catalógo 2
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648"/>
   </bookViews>
   <sheets>
     <sheet name="OMITIDOS" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="206">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -643,6 +643,9 @@
   </si>
   <si>
     <t>MLC4006471046</t>
+  </si>
+  <si>
+    <t>MLC3968074806</t>
   </si>
 </sst>
 </file>
@@ -968,7 +971,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A54"/>
+  <dimension ref="A1:A55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" style="1" bestFit="1" customWidth="1"/>
@@ -1242,6 +1245,11 @@
     <row r="54" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
         <v>204</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A55" s="1" t="s">
+        <v>205</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se configuran publicaciones de catalógo 3
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="OMITIDOS" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="207">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -646,6 +646,9 @@
   </si>
   <si>
     <t>MLC3968074806</t>
+  </si>
+  <si>
+    <t>MLC4087433116</t>
   </si>
 </sst>
 </file>
@@ -971,7 +974,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A55"/>
+  <dimension ref="A1:A56"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" style="1" bestFit="1" customWidth="1"/>
@@ -1250,6 +1253,11 @@
     <row r="55" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
         <v>205</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A56" s="1" t="s">
+        <v>206</v>
       </c>
     </row>
   </sheetData>
@@ -1792,7 +1800,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -1841,7 +1849,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>26</v>
       </c>
@@ -2174,7 +2182,7 @@
   <autoFilter ref="A1:B49">
     <filterColumn colId="0">
       <filters>
-        <filter val="MLC3394755938"/>
+        <filter val="MLC1811410459"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
Se configuran publicaciones de catalógo 4
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="OMITIDOS" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="209">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -652,6 +652,9 @@
   </si>
   <si>
     <t>MLC4333187724</t>
+  </si>
+  <si>
+    <t>MLC3940401778</t>
   </si>
 </sst>
 </file>
@@ -1742,7 +1745,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
@@ -2183,6 +2186,14 @@
         <v>200</v>
       </c>
       <c r="B49">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>208</v>
+      </c>
+      <c r="B50">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Se configuran publicaciones de catalógo 5
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="209">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -1745,7 +1745,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:C50"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
@@ -2181,7 +2181,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="49" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>200</v>
       </c>
@@ -2189,12 +2189,23 @@
         <v>4</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>208</v>
       </c>
       <c r="B50">
         <v>4</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>22</v>
+      </c>
+      <c r="B51">
+        <v>9</v>
+      </c>
+      <c r="C51">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se configuran publicaciones de catalógo 6
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">OMITIDOS!$A$1:$A$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Pack!$A$1:$B$42</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stock ML'!$A$1:$B$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stock ML'!$A$1:$B$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'VARIANTES VALIDAR'!$A$1:$A$54</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="209">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -1745,7 +1745,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
@@ -1811,7 +1811,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -1819,12 +1819,15 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>22</v>
       </c>
       <c r="B9">
-        <v>6</v>
+        <v>9</v>
+      </c>
+      <c r="C9">
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
@@ -2181,7 +2184,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="49" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>200</v>
       </c>
@@ -2189,7 +2192,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>208</v>
       </c>
@@ -2197,22 +2200,11 @@
         <v>4</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A51" t="s">
-        <v>22</v>
-      </c>
-      <c r="B51">
-        <v>9</v>
-      </c>
-      <c r="C51">
-        <v>3</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:B49">
+  <autoFilter ref="A1:B51">
     <filterColumn colId="0">
       <filters>
-        <filter val="MLC1811410459"/>
+        <filter val="MLC3374358846"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
Se configuran publicaciones de catalógo 8
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="209">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -1745,7 +1745,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:C51"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
@@ -1824,10 +1824,7 @@
         <v>22</v>
       </c>
       <c r="B9">
-        <v>9</v>
-      </c>
-      <c r="C9">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
@@ -2184,7 +2181,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="49" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>200</v>
       </c>
@@ -2192,7 +2189,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="50" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>208</v>
       </c>
@@ -2200,7 +2197,18 @@
         <v>4</v>
       </c>
     </row>
-    <row r="51" spans="1:2" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="51" spans="1:3" hidden="1" x14ac:dyDescent="0.3"/>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>18</v>
+      </c>
+      <c r="B52">
+        <v>9</v>
+      </c>
+      <c r="C52">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:B51">
     <filterColumn colId="0">

</xml_diff>

<commit_message>
Se configura kit de transmisión
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="OMITIDOS" sheetId="1" r:id="rId1"/>
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">OMITIDOS!$A$1:$A$49</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Pack!$A$1:$B$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Pack!$A$1:$B$54</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stock ML'!$A$1:$B$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'VARIANTES VALIDAR'!$A$1:$A$54</definedName>
   </definedNames>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="211">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -603,9 +603,6 @@
     <t>MLC4152901046</t>
   </si>
   <si>
-    <t>MLC2928322094</t>
-  </si>
-  <si>
     <t>MLC4229052730</t>
   </si>
   <si>
@@ -655,6 +652,15 @@
   </si>
   <si>
     <t>MLC3940401778</t>
+  </si>
+  <si>
+    <t>MLC14471876954</t>
+  </si>
+  <si>
+    <t>MLC4453960620</t>
+  </si>
+  <si>
+    <t>MLC3400268030</t>
   </si>
 </sst>
 </file>
@@ -1233,17 +1239,17 @@
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.3">
@@ -1253,22 +1259,22 @@
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
   </sheetData>
@@ -1598,7 +1604,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>184</v>
       </c>
@@ -1606,7 +1612,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>184</v>
       </c>
@@ -1630,7 +1636,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>186</v>
       </c>
@@ -1638,7 +1644,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>186</v>
       </c>
@@ -1646,7 +1652,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>186</v>
       </c>
@@ -1659,7 +1665,7 @@
         <v>190</v>
       </c>
       <c r="B46" t="s">
-        <v>191</v>
+        <v>210</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
@@ -1678,59 +1684,59 @@
         <v>189</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
+        <v>192</v>
+      </c>
+      <c r="B49" t="s">
         <v>193</v>
       </c>
-      <c r="B49" t="s">
+    </row>
+    <row r="50" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>192</v>
+      </c>
+      <c r="B50" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A50" t="s">
+    <row r="51" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>195</v>
+      </c>
+      <c r="B51" t="s">
         <v>193</v>
       </c>
-      <c r="B50" t="s">
+    </row>
+    <row r="52" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A51" t="s">
+      <c r="B52" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
         <v>196</v>
-      </c>
-      <c r="B51" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A52" t="s">
-        <v>196</v>
-      </c>
-      <c r="B52" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A53" t="s">
-        <v>197</v>
       </c>
       <c r="B53" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
+        <v>196</v>
+      </c>
+      <c r="B54" t="s">
         <v>197</v>
       </c>
-      <c r="B54" t="s">
-        <v>198</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B42">
+  <autoFilter ref="A1:B54">
     <filterColumn colId="0">
       <filters>
-        <filter val="MLC2018355127"/>
+        <filter val="MLC4152901046"/>
       </filters>
     </filterColumn>
     <sortState ref="A4:B6">
@@ -1745,7 +1751,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:C52"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
@@ -2161,7 +2167,7 @@
     </row>
     <row r="47" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B47">
         <v>12</v>
@@ -2172,7 +2178,7 @@
     </row>
     <row r="48" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B48">
         <v>4</v>
@@ -2183,7 +2189,7 @@
     </row>
     <row r="49" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B49">
         <v>4</v>
@@ -2191,7 +2197,7 @@
     </row>
     <row r="50" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B50">
         <v>4</v>
@@ -2207,6 +2213,28 @@
       </c>
       <c r="C52">
         <v>3</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>208</v>
+      </c>
+      <c r="B53">
+        <v>6</v>
+      </c>
+      <c r="C53">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>209</v>
+      </c>
+      <c r="B54">
+        <v>6</v>
+      </c>
+      <c r="C54">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se configura kit mantención semi + filtro fz16
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="212">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -661,6 +661,9 @@
   </si>
   <si>
     <t>MLC3400268030</t>
+  </si>
+  <si>
+    <t>MLC4460695676</t>
   </si>
 </sst>
 </file>
@@ -1287,7 +1290,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
@@ -1729,6 +1732,22 @@
         <v>196</v>
       </c>
       <c r="B54" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>211</v>
+      </c>
+      <c r="B55" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>211</v>
+      </c>
+      <c r="B56" t="s">
         <v>197</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Se configura discos embrague ybr125
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="OMITIDOS" sheetId="1" r:id="rId1"/>
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">OMITIDOS!$A$1:$A$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Pack!$A$1:$B$54</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stock ML'!$A$1:$B$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stock ML'!$A$1:$B$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'VARIANTES VALIDAR'!$A$1:$A$54</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="213">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -664,6 +664,9 @@
   </si>
   <si>
     <t>MLC4460695676</t>
+  </si>
+  <si>
+    <t>MLC2082076221</t>
   </si>
 </sst>
 </file>
@@ -1770,7 +1773,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
@@ -1844,7 +1847,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -2223,7 +2226,7 @@
       </c>
     </row>
     <row r="51" spans="1:3" hidden="1" x14ac:dyDescent="0.3"/>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>18</v>
       </c>
@@ -2234,7 +2237,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>208</v>
       </c>
@@ -2245,7 +2248,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>209</v>
       </c>
@@ -2256,11 +2259,22 @@
         <v>6</v>
       </c>
     </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>212</v>
+      </c>
+      <c r="B55">
+        <v>8</v>
+      </c>
+      <c r="C55">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B51">
+  <autoFilter ref="A1:B55">
     <filterColumn colId="0">
       <filters>
-        <filter val="MLC3374358846"/>
+        <filter val="MLC2082076221"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
Se prueba quitar configuración de excel 3
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -14,8 +14,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">OMITIDOS!$A$1:$A$49</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Pack!$A$1:$B$54</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stock ML'!$A$1:$B$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Pack!$A$1:$B$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stock ML'!$A$1:$B$54</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'VARIANTES VALIDAR'!$A$1:$A$54</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
@@ -1292,7 +1292,6 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:C56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1308,7 +1307,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>131</v>
       </c>
@@ -1316,7 +1315,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>131</v>
       </c>
@@ -1324,7 +1323,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="4" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>135</v>
       </c>
@@ -1335,7 +1334,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="5" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>135</v>
       </c>
@@ -1346,7 +1345,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="6" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>135</v>
       </c>
@@ -1354,7 +1353,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>32</v>
       </c>
@@ -1362,7 +1361,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>32</v>
       </c>
@@ -1370,7 +1369,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>33</v>
       </c>
@@ -1378,7 +1377,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>33</v>
       </c>
@@ -1386,7 +1385,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>23</v>
       </c>
@@ -1394,7 +1393,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>23</v>
       </c>
@@ -1402,7 +1401,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>24</v>
       </c>
@@ -1410,7 +1409,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>24</v>
       </c>
@@ -1418,7 +1417,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>141</v>
       </c>
@@ -1426,7 +1425,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>141</v>
       </c>
@@ -1434,7 +1433,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>144</v>
       </c>
@@ -1442,7 +1441,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>144</v>
       </c>
@@ -1450,7 +1449,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>147</v>
       </c>
@@ -1458,7 +1457,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="20" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>147</v>
       </c>
@@ -1466,7 +1465,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="21" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>153</v>
       </c>
@@ -1474,7 +1473,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="22" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>153</v>
       </c>
@@ -1482,7 +1481,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="23" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>150</v>
       </c>
@@ -1490,7 +1489,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="24" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>150</v>
       </c>
@@ -1498,7 +1497,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="25" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>156</v>
       </c>
@@ -1506,7 +1505,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="26" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>156</v>
       </c>
@@ -1514,7 +1513,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>161</v>
       </c>
@@ -1522,7 +1521,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="28" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>161</v>
       </c>
@@ -1530,7 +1529,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="29" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>163</v>
       </c>
@@ -1538,7 +1537,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="30" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>163</v>
       </c>
@@ -1546,7 +1545,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>163</v>
       </c>
@@ -1554,7 +1553,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>163</v>
       </c>
@@ -1562,7 +1561,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="33" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>169</v>
       </c>
@@ -1570,7 +1569,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="34" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>169</v>
       </c>
@@ -1578,7 +1577,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="35" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>182</v>
       </c>
@@ -1586,7 +1585,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="36" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>182</v>
       </c>
@@ -1594,7 +1593,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="37" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>183</v>
       </c>
@@ -1602,7 +1601,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="38" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>183</v>
       </c>
@@ -1610,7 +1609,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="39" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>184</v>
       </c>
@@ -1618,7 +1617,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="40" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>184</v>
       </c>
@@ -1626,7 +1625,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>185</v>
       </c>
@@ -1634,7 +1633,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="42" spans="1:2" ht="14.4" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>185</v>
       </c>
@@ -1642,7 +1641,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="43" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>186</v>
       </c>
@@ -1650,7 +1649,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="44" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>186</v>
       </c>
@@ -1658,7 +1657,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="45" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>186</v>
       </c>
@@ -1690,7 +1689,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="49" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>192</v>
       </c>
@@ -1698,7 +1697,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="50" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>192</v>
       </c>
@@ -1706,7 +1705,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="51" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>195</v>
       </c>
@@ -1714,7 +1713,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="52" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>195</v>
       </c>
@@ -1722,7 +1721,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="53" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>196</v>
       </c>
@@ -1730,7 +1729,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="54" spans="1:2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>196</v>
       </c>
@@ -1755,12 +1754,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B54">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="MLC4152901046"/>
-      </filters>
-    </filterColumn>
+  <autoFilter ref="A1:B56">
     <sortState ref="A4:B6">
       <sortCondition descending="1" ref="A1:A34"/>
     </sortState>
@@ -1772,8 +1766,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
@@ -1791,7 +1784,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -1799,7 +1792,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -1807,7 +1800,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -1815,7 +1808,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1823,7 +1816,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -1831,7 +1824,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -1839,7 +1832,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -1847,7 +1840,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -1855,7 +1848,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -1866,7 +1859,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>24</v>
       </c>
@@ -1877,7 +1870,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -1888,7 +1881,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>26</v>
       </c>
@@ -1899,7 +1892,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>27</v>
       </c>
@@ -1907,7 +1900,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>28</v>
       </c>
@@ -1915,7 +1908,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>29</v>
       </c>
@@ -1923,7 +1916,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>30</v>
       </c>
@@ -1931,7 +1924,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>31</v>
       </c>
@@ -1939,7 +1932,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>32</v>
       </c>
@@ -1947,7 +1940,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>34</v>
       </c>
@@ -1958,7 +1951,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>35</v>
       </c>
@@ -1966,7 +1959,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="22" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>36</v>
       </c>
@@ -1974,7 +1967,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>37</v>
       </c>
@@ -1982,7 +1975,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="24" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>38</v>
       </c>
@@ -1990,7 +1983,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>39</v>
       </c>
@@ -1998,7 +1991,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>40</v>
       </c>
@@ -2009,7 +2002,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>41</v>
       </c>
@@ -2017,7 +2010,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>42</v>
       </c>
@@ -2025,7 +2018,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="29" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>43</v>
       </c>
@@ -2033,7 +2026,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="30" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>32</v>
       </c>
@@ -2044,7 +2037,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>155</v>
       </c>
@@ -2052,7 +2045,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="32" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>159</v>
       </c>
@@ -2060,7 +2053,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="33" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>160</v>
       </c>
@@ -2068,7 +2061,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="34" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>162</v>
       </c>
@@ -2079,7 +2072,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="35" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>170</v>
       </c>
@@ -2090,7 +2083,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="36" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>171</v>
       </c>
@@ -2098,7 +2091,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>172</v>
       </c>
@@ -2106,7 +2099,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="38" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>173</v>
       </c>
@@ -2114,7 +2107,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="39" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>174</v>
       </c>
@@ -2122,7 +2115,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="40" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>175</v>
       </c>
@@ -2130,7 +2123,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="41" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>176</v>
       </c>
@@ -2138,7 +2131,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="42" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>177</v>
       </c>
@@ -2146,7 +2139,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="43" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>15</v>
       </c>
@@ -2154,7 +2147,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>178</v>
       </c>
@@ -2165,7 +2158,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="45" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>179</v>
       </c>
@@ -2176,7 +2169,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="46" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>181</v>
       </c>
@@ -2187,7 +2180,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="47" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>191</v>
       </c>
@@ -2198,7 +2191,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="48" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>198</v>
       </c>
@@ -2209,7 +2202,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="49" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>199</v>
       </c>
@@ -2217,7 +2210,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="50" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>207</v>
       </c>
@@ -2225,21 +2218,31 @@
         <v>4</v>
       </c>
     </row>
-    <row r="51" spans="1:3" hidden="1" x14ac:dyDescent="0.3"/>
-    <row r="52" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>18</v>
+      </c>
+      <c r="B51">
+        <v>9</v>
+      </c>
+      <c r="C51">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>18</v>
+        <v>208</v>
       </c>
       <c r="B52">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C52">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B53">
         <v>6</v>
@@ -2248,36 +2251,19 @@
         <v>6</v>
       </c>
     </row>
-    <row r="54" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B54">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C54">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A55" t="s">
-        <v>212</v>
-      </c>
-      <c r="B55">
-        <v>8</v>
-      </c>
-      <c r="C55">
         <v>4</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B55">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="MLC2082076221"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:B55"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="260" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Se configura kit mantención yamalube + filtro yz
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="OMITIDOS" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="215">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -667,6 +667,12 @@
   </si>
   <si>
     <t>MLC2082076221</t>
+  </si>
+  <si>
+    <t>MLC4460694864</t>
+  </si>
+  <si>
+    <t>MLC3940401348</t>
   </si>
 </sst>
 </file>
@@ -1292,7 +1298,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
@@ -1751,6 +1757,22 @@
       </c>
       <c r="B56" t="s">
         <v>197</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>213</v>
+      </c>
+      <c r="B57" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>213</v>
+      </c>
+      <c r="B58" t="s">
+        <v>214</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se configura kit mantención yamalube + filtro fz16
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="216">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -673,6 +673,9 @@
   </si>
   <si>
     <t>MLC3940401348</t>
+  </si>
+  <si>
+    <t>MLC4517123674</t>
   </si>
 </sst>
 </file>
@@ -1298,7 +1301,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
@@ -1773,6 +1776,22 @@
       </c>
       <c r="B58" t="s">
         <v>214</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>215</v>
+      </c>
+      <c r="B59" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>215</v>
+      </c>
+      <c r="B60" t="s">
+        <v>197</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se configura liqui moly street race
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="OMITIDOS" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="220">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -676,6 +676,18 @@
   </si>
   <si>
     <t>MLC4517123674</t>
+  </si>
+  <si>
+    <t>MLC2293144735</t>
+  </si>
+  <si>
+    <t>MLC4587465062</t>
+  </si>
+  <si>
+    <t>MLC4587478054</t>
+  </si>
+  <si>
+    <t>MLC4536477250</t>
   </si>
 </sst>
 </file>
@@ -1001,7 +1013,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A57"/>
+  <dimension ref="A1:A59"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" style="1" bestFit="1" customWidth="1"/>
@@ -1290,6 +1302,16 @@
     <row r="57" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
         <v>206</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A58" s="1" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A59" s="1" t="s">
+        <v>218</v>
       </c>
     </row>
   </sheetData>
@@ -1807,7 +1829,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
@@ -2300,6 +2322,22 @@
         <v>8</v>
       </c>
       <c r="C54">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>216</v>
+      </c>
+      <c r="B55">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>219</v>
+      </c>
+      <c r="B56">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Se configuran discos de embrague xtz125
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">OMITIDOS!$A$1:$A$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Pack!$A$1:$B$56</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stock ML'!$A$1:$B$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Stock ML'!$A$1:$B$59</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'VARIANTES VALIDAR'!$A$1:$A$54</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="223">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -691,6 +691,12 @@
   </si>
   <si>
     <t>MLC1663480753</t>
+  </si>
+  <si>
+    <t>MLC2223320367</t>
+  </si>
+  <si>
+    <t>MLC4093496418</t>
   </si>
 </sst>
 </file>
@@ -1832,7 +1838,8 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C57"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
@@ -1850,7 +1857,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>14</v>
       </c>
@@ -1858,7 +1865,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -1866,7 +1873,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -1874,7 +1881,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1882,7 +1889,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>19</v>
       </c>
@@ -1890,7 +1897,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -1898,7 +1905,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -1906,7 +1913,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -1914,7 +1921,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -1925,7 +1932,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>24</v>
       </c>
@@ -1936,7 +1943,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -1947,7 +1954,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>26</v>
       </c>
@@ -1958,7 +1965,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>27</v>
       </c>
@@ -1966,7 +1973,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>28</v>
       </c>
@@ -1974,7 +1981,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>29</v>
       </c>
@@ -1982,7 +1989,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>30</v>
       </c>
@@ -1990,7 +1997,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>31</v>
       </c>
@@ -1998,7 +2005,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>32</v>
       </c>
@@ -2006,7 +2013,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>34</v>
       </c>
@@ -2017,7 +2024,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>35</v>
       </c>
@@ -2025,7 +2032,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>36</v>
       </c>
@@ -2033,7 +2040,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>37</v>
       </c>
@@ -2041,7 +2048,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>38</v>
       </c>
@@ -2049,7 +2056,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>39</v>
       </c>
@@ -2057,7 +2064,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>40</v>
       </c>
@@ -2068,7 +2075,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>41</v>
       </c>
@@ -2076,7 +2083,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>42</v>
       </c>
@@ -2084,7 +2091,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>43</v>
       </c>
@@ -2092,7 +2099,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>32</v>
       </c>
@@ -2103,7 +2110,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>155</v>
       </c>
@@ -2111,7 +2118,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>159</v>
       </c>
@@ -2119,7 +2126,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>160</v>
       </c>
@@ -2127,7 +2134,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>162</v>
       </c>
@@ -2138,7 +2145,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>170</v>
       </c>
@@ -2149,7 +2156,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>171</v>
       </c>
@@ -2157,7 +2164,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>172</v>
       </c>
@@ -2165,7 +2172,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>173</v>
       </c>
@@ -2173,7 +2180,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>174</v>
       </c>
@@ -2181,7 +2188,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>175</v>
       </c>
@@ -2189,7 +2196,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>176</v>
       </c>
@@ -2197,7 +2204,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>177</v>
       </c>
@@ -2205,7 +2212,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>15</v>
       </c>
@@ -2213,7 +2220,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>178</v>
       </c>
@@ -2224,7 +2231,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>179</v>
       </c>
@@ -2235,7 +2242,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>181</v>
       </c>
@@ -2246,7 +2253,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>191</v>
       </c>
@@ -2257,7 +2264,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>198</v>
       </c>
@@ -2268,7 +2275,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>199</v>
       </c>
@@ -2276,7 +2283,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>207</v>
       </c>
@@ -2284,7 +2291,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>18</v>
       </c>
@@ -2295,7 +2302,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>208</v>
       </c>
@@ -2306,7 +2313,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>209</v>
       </c>
@@ -2317,7 +2324,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>212</v>
       </c>
@@ -2328,7 +2335,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>216</v>
       </c>
@@ -2336,7 +2343,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>219</v>
       </c>
@@ -2344,7 +2351,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>220</v>
       </c>
@@ -2352,8 +2359,33 @@
         <v>5</v>
       </c>
     </row>
+    <row r="58" spans="1:3" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>221</v>
+      </c>
+      <c r="B58">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>222</v>
+      </c>
+      <c r="B59">
+        <v>8</v>
+      </c>
+      <c r="C59">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B55"/>
+  <autoFilter ref="A1:B59">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="MLC4093496418"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="260" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Se configura kit mantención liqui moly 10w40 + filtro hiflo hf140
</commit_message>
<xml_diff>
--- a/validar-ml/configuracion.xlsx
+++ b/validar-ml/configuracion.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="OMITIDOS" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="226">
   <si>
     <t>Número Publicación</t>
   </si>
@@ -697,6 +697,15 @@
   </si>
   <si>
     <t>MLC4093496418</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MLC4545934758 </t>
+  </si>
+  <si>
+    <t>MLC2295040215</t>
+  </si>
+  <si>
+    <t>MLC2012989525</t>
   </si>
 </sst>
 </file>
@@ -1332,7 +1341,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C62"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.6640625" bestFit="1" customWidth="1"/>
@@ -1823,6 +1832,22 @@
       </c>
       <c r="B60" t="s">
         <v>197</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>223</v>
+      </c>
+      <c r="B61" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>223</v>
+      </c>
+      <c r="B62" t="s">
+        <v>225</v>
       </c>
     </row>
   </sheetData>

</xml_diff>